<commit_message>
Fix: Actualizar correo de usuario CASA CHANALUISA ALEX WLADIMIR a acasa@quito-turismo.gob.ec
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/sitra2026.xlsx
+++ b/doc/sitra2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acasa\Documents\Desarrollo\Sis_asignacion de memos\v2\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://quitoturismo365-my.sharepoint.com/personal/acasa_quito-turismo_gob_ec/Documents/Documentos/Desarrollo/Sis_asignacion de memos/seguimiento_sitra/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C775F9D-7ABE-427B-9A51-979B4E6CC4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{6C775F9D-7ABE-427B-9A51-979B4E6CC4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE532FB1-CFE9-4810-A14C-0DED5153666A}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1859918A-2E0A-4C66-A4C1-5BE39778083C}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1859918A-2E0A-4C66-A4C1-5BE39778083C}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasignados" sheetId="1" r:id="rId1"/>
@@ -286,7 +286,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -394,12 +394,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -738,17 +738,20 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.85546875" customWidth="1"/>
     <col min="4" max="4" width="34.5703125" customWidth="1"/>
     <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.140625" style="17" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="4.140625" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" customWidth="1"/>
     <col min="9" max="9" width="63.28515625" customWidth="1"/>
     <col min="10" max="10" width="32.42578125" customWidth="1"/>
-    <col min="11" max="11" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" customWidth="1"/>
+    <col min="12" max="12" width="22.5703125" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>